<commit_message>
Memo update pack; team model v2 ADR display table fix; memo inputs for the rewrite
- deck/MEMO_UPDATE_2026-09-29.md: every v2 number (quarterly, FY, valuation build, nights
  decomposition, margin bridge), line-by-line memo replacements, known workbook issues
  (Cover E35 -$0.70, Cover "2Q27" columns showing 3Q27 revenue/nights, market cap), chart
  index and file index, for a memo rewrite that only sees GitHub.
- model/Caimanes_Citadel_ABNB_Model_v2.xlsx: ADR_Engine rows 120-129 GBV now live formulas
  (model nights x each rule's ADR); they were frozen at v1 nights. Nothing else reads them.
- model/ABNB Citadel Pitch Memo.docx/.pdf (24 Sep, v1 numbers), deck/drafts thesis 1-3
  drafts and two_pager_cuts, deck/Graphs originals: committed unchanged as inputs.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0151H91mtdwA2sNaCPdY2Qct
</commit_message>
<xml_diff>
--- a/model/Caimanes_Citadel_ABNB_Model_v2.xlsx
+++ b/model/Caimanes_Citadel_ABNB_Model_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krish\citadel-abnb\model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krish\citadel-abnb\.worktrees\charts\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C948937-46C4-4097-805F-BFD6DDBEDE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EDB2E9-8993-4D8D-90E4-0063597D3427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -878,9 +878,6 @@
     <t>rule</t>
   </si>
   <si>
-    <t>quarter → ex-FX (pp) | ADR ($) | GBV ($bn)</t>
-  </si>
-  <si>
     <t>3Q26</t>
   </si>
   <si>
@@ -1716,6 +1713,9 @@
   </si>
   <si>
     <t xml:space="preserve">  RNPL cancellations (pp) — cohort engine central cell (management-implied +6pt RNPL cancel rate, 25% rebooked, lead 2.2, ADR +25%): 3Q26 −0.93, 4Q26 −0.85 (overnight2 D1); 2027 = n02 base tail shape × 1.566 (4Q26 ratio)</t>
+  </si>
+  <si>
+    <t>quarter → ex-FX (pp) | ADR ($) | GBV ($bn; = model nights × this rule's ADR, live formula since v2)</t>
   </si>
 </sst>
 </file>
@@ -5611,7 +5611,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32.4" x14ac:dyDescent="0.3">
       <c r="A1" s="86" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B1" s="85"/>
       <c r="C1" s="85"/>
@@ -5644,7 +5644,7 @@
       <c r="L2" s="85"/>
       <c r="M2" s="85"/>
       <c r="O2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="P2">
         <v>151.38999999999999</v>
@@ -5668,7 +5668,7 @@
       <c r="L3" s="85"/>
       <c r="M3" s="85"/>
       <c r="O3" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="P3">
         <v>589.6</v>
@@ -5713,7 +5713,7 @@
         <v>30</v>
       </c>
       <c r="O4" s="89" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="P4" s="90">
         <f>P2*P3</f>
@@ -5722,7 +5722,7 @@
     </row>
     <row r="5" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A5" s="62" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B5" s="55">
         <f>Income_Statement!J11</f>
@@ -5773,7 +5773,7 @@
         <v>3309.1926097535961</v>
       </c>
       <c r="O5" s="54" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="P5" s="54">
         <v>2476</v>
@@ -5781,7 +5781,7 @@
     </row>
     <row r="6" spans="1:16" s="54" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="64" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B6" s="65">
         <f>Income_Statement!J12</f>
@@ -5832,7 +5832,7 @@
         <v>7.4860074235129304E-2</v>
       </c>
       <c r="O6" s="54" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="P6" s="54">
         <v>12069</v>
@@ -5840,7 +5840,7 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="66" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B7" s="67">
         <f>Income_Statement!J4</f>
@@ -5891,7 +5891,7 @@
         <v>138.51630796221002</v>
       </c>
       <c r="O7" s="89" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="P7" s="90">
         <f>P4+P5-P6</f>
@@ -5900,7 +5900,7 @@
     </row>
     <row r="8" spans="1:16" s="54" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="64" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B8" s="68">
         <f>Income_Statement!J5</f>
@@ -5953,7 +5953,7 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="66" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B9" s="67">
         <f>Income_Statement!J9</f>
@@ -6008,7 +6008,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="64" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B10" s="69">
         <f>Income_Statement!J10</f>
@@ -6062,7 +6062,7 @@
     </row>
     <row r="11" spans="1:16" s="54" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="75" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B11" s="76">
         <f>Income_Statement!J13</f>
@@ -6127,7 +6127,7 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="62" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B13" s="55">
         <f>Income_Statement!J20</f>
@@ -6180,7 +6180,7 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="62" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B14" s="55">
         <f>Income_Statement!J23</f>
@@ -6233,7 +6233,7 @@
     </row>
     <row r="15" spans="1:16" s="54" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="64" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B15" s="68">
         <f>Income_Statement!J23/Income_Statement!F23-1</f>
@@ -6286,7 +6286,7 @@
     </row>
     <row r="16" spans="1:16" s="54" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="75" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B16" s="76">
         <f>B14/B5</f>
@@ -6348,7 +6348,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="62" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B18" s="55">
         <f>Income_Statement!J27</f>
@@ -6401,7 +6401,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="62" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B19" s="55">
         <f>Income_Statement!J33</f>
@@ -6454,7 +6454,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="70" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B20" s="71">
         <f>Income_Statement!J35</f>
@@ -6508,74 +6508,74 @@
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="59"/>
       <c r="B22" s="60" t="s">
+        <v>538</v>
+      </c>
+      <c r="C22" s="60" t="s">
         <v>539</v>
       </c>
-      <c r="C22" s="60" t="s">
-        <v>540</v>
-      </c>
       <c r="D22" s="60" t="s">
+        <v>538</v>
+      </c>
+      <c r="E22" s="60" t="s">
         <v>539</v>
       </c>
-      <c r="E22" s="60" t="s">
-        <v>540</v>
-      </c>
       <c r="F22" s="60" t="s">
+        <v>538</v>
+      </c>
+      <c r="G22" s="60" t="s">
         <v>539</v>
       </c>
-      <c r="G22" s="60" t="s">
-        <v>540</v>
-      </c>
       <c r="H22" s="60" t="s">
+        <v>538</v>
+      </c>
+      <c r="I22" s="60" t="s">
         <v>539</v>
       </c>
-      <c r="I22" s="60" t="s">
-        <v>540</v>
-      </c>
       <c r="J22" s="60" t="s">
+        <v>538</v>
+      </c>
+      <c r="K22" s="61" t="s">
         <v>539</v>
-      </c>
-      <c r="K22" s="61" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="81" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B23" s="82" t="s">
+        <v>280</v>
+      </c>
+      <c r="C23" s="82" t="s">
+        <v>280</v>
+      </c>
+      <c r="D23" s="82" t="s">
         <v>281</v>
       </c>
-      <c r="C23" s="82" t="s">
+      <c r="E23" s="82" t="s">
         <v>281</v>
       </c>
-      <c r="D23" s="82" t="s">
+      <c r="F23" s="82" t="s">
         <v>282</v>
       </c>
-      <c r="E23" s="82" t="s">
+      <c r="G23" s="82" t="s">
         <v>282</v>
       </c>
-      <c r="F23" s="82" t="s">
+      <c r="H23" s="82" t="s">
         <v>283</v>
       </c>
-      <c r="G23" s="82" t="s">
+      <c r="I23" s="82" t="s">
         <v>283</v>
       </c>
-      <c r="H23" s="82" t="s">
-        <v>284</v>
-      </c>
-      <c r="I23" s="82" t="s">
-        <v>284</v>
-      </c>
       <c r="J23" s="82" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="K23" s="83" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A24" s="62" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B24" s="55">
         <f>H5</f>
@@ -6620,7 +6620,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="64" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B25" s="84">
         <f>B24/C24-1</f>
@@ -6650,7 +6650,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="62" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B26" s="88">
         <f>H7</f>
@@ -6684,7 +6684,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="62" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B27" s="67">
         <f>H9</f>
@@ -6717,7 +6717,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="62" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B28" s="55">
         <f>H14</f>
@@ -6762,7 +6762,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="70" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B29" s="71">
         <f>H20</f>
@@ -6802,24 +6802,24 @@
     </row>
     <row r="31" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="72" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B31" s="95" t="s">
+        <v>555</v>
+      </c>
+      <c r="C31" s="96" t="s">
+        <v>536</v>
+      </c>
+      <c r="D31" s="96" t="s">
         <v>556</v>
       </c>
-      <c r="C31" s="96" t="s">
-        <v>537</v>
-      </c>
-      <c r="D31" s="96" t="s">
-        <v>557</v>
-      </c>
       <c r="E31" s="114" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A32" s="62" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B32" s="91">
         <f>P7/SUM(H14:K14)</f>
@@ -6840,7 +6840,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="62" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B33" s="91">
         <f>P7/D28</f>
@@ -6861,7 +6861,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="70" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B34" s="93">
         <f>P7/J28</f>
@@ -6914,7 +6914,7 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7008,16 +7008,16 @@
       </c>
       <c r="V3" s="4"/>
       <c r="W3" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="X3" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="X3" s="6" t="s">
+      <c r="Y3" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="Y3" s="6" t="s">
+      <c r="Z3" s="6" t="s">
         <v>350</v>
-      </c>
-      <c r="Z3" s="6" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
@@ -7220,7 +7220,7 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -7250,7 +7250,7 @@
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B7" s="15">
         <f t="shared" ref="B7:U7" si="3">B4*B9/1000</f>
@@ -7404,7 +7404,7 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B9" s="19">
         <f>ADR_Engine!K6</f>
@@ -7574,7 +7574,7 @@
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B11" s="30">
         <v>1818</v>
@@ -7742,7 +7742,7 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B13" s="33">
         <f t="shared" ref="B13:O13" si="14">B11/(B7*1000)</f>
@@ -7837,7 +7837,7 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B15" s="30">
         <v>428</v>
@@ -7924,7 +7924,7 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B16" s="30">
         <v>267</v>
@@ -8011,7 +8011,7 @@
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B17" s="30">
         <v>271</v>
@@ -8098,7 +8098,7 @@
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B18" s="30">
         <v>422</v>
@@ -8185,7 +8185,7 @@
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B19" s="30">
         <v>191</v>
@@ -8272,7 +8272,7 @@
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B20" s="31">
         <f t="shared" ref="B20:S20" si="22">SUM(B15:B19)</f>
@@ -8373,7 +8373,7 @@
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B21" s="9">
         <f t="shared" ref="B21:S21" si="23">B20/B11</f>
@@ -8474,7 +8474,7 @@
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B22" s="30">
         <v>11</v>
@@ -8561,7 +8561,7 @@
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B23" s="30">
         <v>262</v>
@@ -8648,7 +8648,7 @@
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B24" s="9">
         <f t="shared" ref="B24:S24" si="26">B23/B11</f>
@@ -8827,7 +8827,7 @@
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B26" s="30">
         <v>240</v>
@@ -8914,7 +8914,7 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B27" s="30">
         <v>-5</v>
@@ -9001,7 +9001,7 @@
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B28" s="30">
         <v>146</v>
@@ -9088,7 +9088,7 @@
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B29" s="30">
         <v>4</v>
@@ -9175,7 +9175,7 @@
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B30" s="30">
         <v>-7</v>
@@ -9262,7 +9262,7 @@
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B31" s="30">
         <v>130</v>
@@ -9349,7 +9349,7 @@
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B32" s="30">
         <v>13.4</v>
@@ -9436,7 +9436,7 @@
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B33" s="30">
         <v>117</v>
@@ -9523,7 +9523,7 @@
     </row>
     <row r="34" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B34" s="8">
         <v>670</v>
@@ -9607,7 +9607,7 @@
     </row>
     <row r="35" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B35" s="10">
         <v>0.18</v>
@@ -9691,7 +9691,7 @@
     </row>
     <row r="37" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -9721,7 +9721,7 @@
     </row>
     <row r="38" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="P38" s="30">
         <v>4744.32</v>
@@ -9744,7 +9744,7 @@
     </row>
     <row r="39" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="P39" s="32">
         <f t="shared" ref="P39:S39" si="40">P11/P38-1</f>
@@ -9773,7 +9773,7 @@
     </row>
     <row r="40" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="P40" s="30">
         <v>2361.52</v>
@@ -9796,7 +9796,7 @@
     </row>
     <row r="41" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="P41" s="32">
         <f t="shared" ref="P41:S41" si="41">P23/P40-1</f>
@@ -9825,7 +9825,7 @@
     </row>
     <row r="42" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="P42" s="31">
         <f>P11*0.503668738501203</f>
@@ -9854,7 +9854,7 @@
     </row>
     <row r="43" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P43" s="31">
         <f t="shared" ref="P43:S43" si="42">P42-P23</f>
@@ -9883,7 +9883,7 @@
     </row>
     <row r="44" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="P44" s="30">
         <v>15.20793246038539</v>
@@ -9906,7 +9906,7 @@
     </row>
     <row r="46" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A46" s="41" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B46" s="43"/>
       <c r="C46" s="43"/>
@@ -9931,12 +9931,12 @@
     </row>
     <row r="47" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A47" s="45" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="48" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A48" s="44" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B48" s="10">
         <v>3.65</v>
@@ -9944,7 +9944,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="44" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B49" s="10">
         <v>3.6</v>
@@ -9952,7 +9952,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="44" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B50" s="10">
         <v>3.7</v>
@@ -9960,7 +9960,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="44" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B51" s="10">
         <v>3.65</v>
@@ -9968,7 +9968,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="44" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B52" s="10">
         <v>1.7</v>
@@ -9976,7 +9976,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="44" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B53" s="8">
         <v>1</v>
@@ -9984,7 +9984,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="44" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B54" s="11">
         <v>0.29714329912855497</v>
@@ -9992,7 +9992,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="44" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B55" s="10">
         <v>0.72</v>
@@ -10000,7 +10000,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" s="44" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B56" s="10">
         <v>0</v>
@@ -10008,7 +10008,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" s="44" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B57" s="30">
         <v>224</v>
@@ -10016,7 +10016,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" s="44" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B58" s="30">
         <v>30</v>
@@ -10024,7 +10024,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" s="44" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B59" s="30">
         <v>330</v>
@@ -10032,7 +10032,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" s="44" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B60" s="10">
         <v>0.36</v>
@@ -10040,7 +10040,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" s="44" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B61" s="11">
         <v>0.215</v>
@@ -10048,7 +10048,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" s="44" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B62" s="8">
         <v>-14</v>
@@ -10056,7 +10056,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="44" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B63" s="8">
         <v>-10</v>
@@ -10064,7 +10064,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" s="44" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B64" s="8">
         <v>8</v>
@@ -10072,7 +10072,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="44" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B65" s="8">
         <v>0</v>
@@ -10080,7 +10080,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="44" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B66" s="8">
         <v>9</v>
@@ -10088,7 +10088,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" s="44" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B67" s="8">
         <v>8</v>
@@ -10096,7 +10096,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" s="44" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B68" s="30">
         <v>30</v>
@@ -10104,7 +10104,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="44" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B69" s="30">
         <v>1595</v>
@@ -10112,7 +10112,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" s="44" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B70" s="10">
         <v>0.51</v>
@@ -10120,7 +10120,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" s="44" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B71" s="8">
         <v>32</v>
@@ -10128,7 +10128,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" s="44" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B72" s="8">
         <v>25</v>
@@ -10136,7 +10136,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" s="44" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B73" s="8">
         <v>15</v>
@@ -10144,7 +10144,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="44" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B74" s="30">
         <v>781</v>
@@ -10152,7 +10152,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" s="44" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B75" s="8">
         <v>18</v>
@@ -10160,7 +10160,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" s="44" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B76" s="8">
         <v>11</v>
@@ -10168,7 +10168,7 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" s="44" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B77" s="8">
         <v>5</v>
@@ -10176,7 +10176,7 @@
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" s="44" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B78" s="8">
         <v>5</v>
@@ -10184,7 +10184,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" s="44" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B79" s="30">
         <v>0</v>
@@ -10192,7 +10192,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" s="44" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B80" s="46">
         <v>1</v>
@@ -10200,7 +10200,7 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" s="44" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B81" s="30">
         <v>4730</v>
@@ -10208,7 +10208,7 @@
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" s="44" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B82" s="8">
         <v>-0.5</v>
@@ -10216,7 +10216,7 @@
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" s="44" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B83" s="11">
         <v>146.81299999999999</v>
@@ -10224,7 +10224,7 @@
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" s="44" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B84" s="11">
         <v>26.027999999999999</v>
@@ -10232,7 +10232,7 @@
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" s="44" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B85" s="10">
         <v>0.7</v>
@@ -10240,7 +10240,7 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" s="44" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B86" s="8">
         <v>20.633970599907517</v>
@@ -10248,7 +10248,7 @@
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" s="44" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B87" s="10">
         <v>13.177740767185675</v>
@@ -10256,7 +10256,7 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" s="44" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B88" s="11">
         <v>0.8764975067193741</v>
@@ -10264,7 +10264,7 @@
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" s="44" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B89" s="10">
         <v>3.76</v>
@@ -10272,7 +10272,7 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" s="44" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B90" s="30">
         <v>12069</v>
@@ -10280,7 +10280,7 @@
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" s="44" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B91" s="8">
         <v>0</v>
@@ -10288,7 +10288,7 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" s="44" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B92" s="8">
         <v>37</v>
@@ -10296,7 +10296,7 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" s="44" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B93" s="8">
         <v>3.7</v>
@@ -10304,7 +10304,7 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" s="44" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B94" s="8">
         <v>18</v>
@@ -10312,7 +10312,7 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" s="44" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B95" s="8">
         <v>17.5</v>
@@ -10320,7 +10320,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" s="44" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B96" s="8">
         <v>597</v>
@@ -10328,7 +10328,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A97" s="44" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B97" s="11">
         <v>-5.324186618094461</v>
@@ -10336,12 +10336,12 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A99" s="47" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A100" s="44" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="P100" s="11">
         <v>1.0349999999999999</v>
@@ -10364,7 +10364,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A101" s="44" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="P101" s="25">
         <v>0.24590000000000001</v>
@@ -10387,7 +10387,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A102" s="44" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="P102" s="25">
         <v>0.23699999999999999</v>
@@ -10410,7 +10410,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A103" s="44" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="P103" s="25">
         <v>0.24560000000000001</v>
@@ -10433,12 +10433,12 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A105" s="47" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A106" s="44" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B106" s="48">
         <f>$B$69*$B$70*(1+$B$71/100)</f>
@@ -10447,7 +10447,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A107" s="44" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B107" s="48">
         <f>$B$69*(1-$B$70)*(1+$B$72/100)</f>
@@ -10456,7 +10456,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A108" s="44" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B108" s="48">
         <f>N18+O18-$B$106</f>
@@ -10465,7 +10465,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A109" s="44" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B109" s="48">
         <f>$B$74*(1+$B$75/100)</f>
@@ -10474,7 +10474,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A110" s="44" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B110" s="48">
         <f>$B$109-$B$108</f>
@@ -10483,7 +10483,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A111" s="44" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B111" s="48">
         <f>$B$109*(1+$B$76/100)</f>
@@ -10492,7 +10492,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A112" s="44" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B112" s="48">
         <f>(L17+M17)*(1+$B$66/100)</f>
@@ -10501,7 +10501,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A113" s="44" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B113" s="48">
         <f>(N17+O17+$B$112)*(1+$B$67/100)+$B$68</f>
@@ -10510,7 +10510,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A114" s="44" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B114" s="48">
         <f>(L19+M19)*(1+$B$77/100)</f>
@@ -10519,7 +10519,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A115" s="44" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B115" s="48">
         <f>(N19+O19+$B$114)*(1+$B$78/100)</f>
@@ -10528,7 +10528,7 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A116" s="44" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B116" s="48">
         <f>$B$83/$B$48</f>
@@ -10537,7 +10537,7 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A117" s="44" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B117" s="48">
         <f>($B$52+$B$53*$B$54/100)*$P$100/100*$B$84*1000+$B$55*$B$116+($B$57/2+$B$58)/2+$B$60*$B$83</f>
@@ -10546,7 +10546,7 @@
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A118" s="44" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B118" s="48">
         <f>L16*($B$61*(1+$B$62/100)*$B$116/(L4/$B$50)+(1-$B$61)*(1+$B$64/100))</f>
@@ -10555,7 +10555,7 @@
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A119" s="44" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B119" s="48">
         <f>$B$112*$P$101/($P$101+$Q$101)+($B$107+$B$110)*$P$102/($P$102+$Q$102)+$B$114*$P$103/($P$103+$Q$103)</f>
@@ -10564,7 +10564,7 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A120" s="44" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B120" s="48">
         <f>$B$117+$B$118+$B$119</f>
@@ -10573,7 +10573,7 @@
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A121" s="44" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B121" s="48">
         <f>$B$81*(1-(L24*100+$B$82)/100)+$B$86</f>
@@ -10582,7 +10582,7 @@
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A122" s="44" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B122" s="48">
         <f>IF($B$80&gt;=0.5,MAX(0,$B$121-$B$120),0)</f>
@@ -10591,7 +10591,7 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A123" s="44" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B123" s="48">
         <f>$B$122*$B$85</f>
@@ -10600,7 +10600,7 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A124" s="44" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B124" s="48">
         <f>$B$58+$B$122*(1-$B$85)*2</f>
@@ -10609,7 +10609,7 @@
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A125" s="44" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B125" s="48">
         <f>($B$106+$B$107+$B$123)*(1+$B$73/100)</f>
@@ -10618,12 +10618,12 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A127" s="47" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A128" s="44" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="P128" s="14">
         <f>P4/$B$48</f>
@@ -10652,7 +10652,7 @@
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A129" s="44" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="P129" s="15">
         <f t="shared" ref="P129:U129" si="43">($B$52+$B$53*$B$54/100)*P100</f>
@@ -10681,7 +10681,7 @@
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A130" s="44" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="P130" s="48">
         <f t="shared" ref="P130:U130" si="44">P129/100*P7*1000</f>
@@ -10710,7 +10710,7 @@
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A131" s="44" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="P131" s="48">
         <f t="shared" ref="P131:U131" si="45">($B$55+$B$56)*P128</f>
@@ -10739,7 +10739,7 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A132" s="44" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="P132" s="48">
         <f>($B$57/2+$B$124)/2</f>
@@ -10768,7 +10768,7 @@
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A133" s="44" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="P133" s="48">
         <f t="shared" ref="P133:U133" si="46">$B$60*P4</f>
@@ -10797,7 +10797,7 @@
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A134" s="47" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="P134" s="48">
         <f t="shared" ref="P134:U134" si="47">SUM(P130:P133)</f>
@@ -10826,7 +10826,7 @@
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A135" s="44" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="P135" s="49">
         <f t="shared" ref="P135:U135" si="48">L16</f>
@@ -10855,7 +10855,7 @@
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A136" s="44" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="P136" s="14">
         <f>L4/$B$50</f>
@@ -10884,7 +10884,7 @@
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A137" s="44" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="P137" s="48">
         <f>P135*$B$61*(1+$B$62/100)*P128/P136</f>
@@ -10913,7 +10913,7 @@
     </row>
     <row r="138" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A138" s="44" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="P138" s="48">
         <f t="shared" ref="P138:U138" si="49">P135*(1-$B$61)*(1+$B$64/100)</f>
@@ -10942,7 +10942,7 @@
     </row>
     <row r="139" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A139" s="47" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="P139" s="48">
         <f t="shared" ref="P139:U139" si="50">(P137+P138)*(1+$B$65/100)</f>
@@ -10971,7 +10971,7 @@
     </row>
     <row r="140" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A140" s="47" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="P140" s="48">
         <f>$B$112*P101/($P$101+$Q$101)</f>
@@ -11000,7 +11000,7 @@
     </row>
     <row r="141" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A141" s="44" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="P141" s="48">
         <f>$B$107*P102/($P$102+$Q$102)+$B$123</f>
@@ -11029,7 +11029,7 @@
     </row>
     <row r="142" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A142" s="44" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="P142" s="48">
         <f>$B$110*P102/($P$102+$Q$102)</f>
@@ -11058,7 +11058,7 @@
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A143" s="47" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="P143" s="48">
         <f t="shared" ref="P143:U143" si="51">P141+P142</f>
@@ -11087,7 +11087,7 @@
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A144" s="47" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="P144" s="48">
         <f>$B$114*P103/($P$103+$Q$103)</f>
@@ -11116,7 +11116,7 @@
     </row>
     <row r="145" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A145" s="47" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="P145" s="48">
         <f t="shared" ref="P145:U145" si="52">L26*(1+$B$87/100)</f>
@@ -11145,7 +11145,7 @@
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A146" s="44" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="L146" s="30">
         <v>7209</v>
@@ -11186,7 +11186,7 @@
     </row>
     <row r="147" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A147" s="44" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="O147" s="31">
         <f t="shared" ref="O147:U147" si="54">O146*(1-$B$91/100)</f>
@@ -11219,7 +11219,7 @@
     </row>
     <row r="148" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A148" s="47" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="P148" s="48">
         <f t="shared" ref="P148:U148" si="55">$B$88*$B$89/100*($B$90+(P147+O147)/2)/4</f>
@@ -11248,7 +11248,7 @@
     </row>
     <row r="149" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A149" s="47" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="P149" s="21">
         <f>$B$96+$B$97</f>
@@ -11277,12 +11277,12 @@
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A151" s="47" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="152" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A152" s="44" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="P152" s="9">
         <f t="shared" ref="P152:U152" si="56">P24</f>
@@ -11311,7 +11311,7 @@
     </row>
     <row r="153" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A153" s="44" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="P153" s="9">
         <f t="shared" ref="P153:U153" si="57">P40/P38</f>
@@ -11340,7 +11340,7 @@
     </row>
     <row r="154" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A154" s="44" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="P154" s="14">
         <f t="shared" ref="P154:U154" si="58">(P152-P153)*100</f>
@@ -11369,7 +11369,7 @@
     </row>
     <row r="155" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A155" s="44" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="P155" s="32">
         <f t="shared" ref="P155:U155" si="59">P20/L20-1</f>
@@ -11398,7 +11398,7 @@
     </row>
     <row r="156" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A156" s="44" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="P156" s="32">
         <f t="shared" ref="P156:U156" si="60">P18/P11</f>
@@ -11427,7 +11427,7 @@
     </row>
     <row r="157" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A157" s="44" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="P157" s="32">
         <f t="shared" ref="P157:U157" si="61">(P23-L23)/(P11-L11)</f>
@@ -11456,7 +11456,7 @@
     </row>
     <row r="158" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A158" s="44" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
   </sheetData>
@@ -12480,7 +12480,7 @@
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.3">
       <c r="W19" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.3">
@@ -13758,7 +13758,7 @@
     </row>
     <row r="77" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B77" s="117">
         <v>9.1999999999999993</v>
@@ -13895,27 +13895,27 @@
         <v>97</v>
       </c>
       <c r="X83" s="16">
-        <f>SUM(X79:X82)+X91</f>
+        <f t="shared" ref="X83:AC83" si="11">SUM(X79:X82)+X91</f>
         <v>9.1999999999999993</v>
       </c>
       <c r="Y83" s="16">
-        <f>SUM(Y79:Y82)+Y91</f>
+        <f t="shared" si="11"/>
         <v>7.2710000000000008</v>
       </c>
       <c r="Z83" s="16">
-        <f>SUM(Z79:Z82)+Z91</f>
+        <f t="shared" si="11"/>
         <v>7.82</v>
       </c>
       <c r="AA83" s="16">
-        <f>SUM(AA79:AA82)+AA91</f>
+        <f t="shared" si="11"/>
         <v>5.7200000000000006</v>
       </c>
       <c r="AB83" s="16">
-        <f>SUM(AB79:AB82)+AB91</f>
+        <f t="shared" si="11"/>
         <v>6.093</v>
       </c>
       <c r="AC83" s="16">
-        <f>SUM(AC79:AC82)+AC91</f>
+        <f t="shared" si="11"/>
         <v>5.9289999999999994</v>
       </c>
     </row>
@@ -14046,7 +14046,7 @@
     </row>
     <row r="91" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="X91" s="117">
         <v>-0.93</v>
@@ -14199,59 +14199,59 @@
         <v>112</v>
       </c>
       <c r="J95" s="14">
-        <f t="shared" ref="J95:W95" si="11">J93-J94</f>
+        <f t="shared" ref="J95:W95" si="12">J93-J94</f>
         <v>5.68</v>
       </c>
       <c r="K95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6.1300000000000008</v>
       </c>
       <c r="L95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2.91</v>
       </c>
       <c r="M95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>5.92</v>
       </c>
       <c r="N95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-0.1899999999999995</v>
       </c>
       <c r="O95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.67999999999999972</v>
       </c>
       <c r="P95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.1099999999999994</v>
       </c>
       <c r="Q95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-0.3100000000000005</v>
       </c>
       <c r="R95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>4.879999999999999</v>
       </c>
       <c r="S95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-1.8499999999999996</v>
       </c>
       <c r="T95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-4.09</v>
       </c>
       <c r="U95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-8.0500000000000007</v>
       </c>
       <c r="V95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-18.809999999999999</v>
       </c>
       <c r="W95" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>-16.649999999999999</v>
       </c>
     </row>
@@ -14451,59 +14451,59 @@
         <v>128</v>
       </c>
       <c r="J111" s="14">
-        <f t="shared" ref="J111:W111" si="12">J7*100</f>
+        <f t="shared" ref="J111:W111" si="13">J7*100</f>
         <v>18.609206660137122</v>
       </c>
       <c r="K111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>10.993249758919955</v>
       </c>
       <c r="L111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>13.54062186559679</v>
       </c>
       <c r="M111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>12.01814058956916</v>
       </c>
       <c r="N111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>9.4962840627580434</v>
       </c>
       <c r="O111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8.6880973066898459</v>
       </c>
       <c r="P111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8.4805653710247277</v>
       </c>
       <c r="Q111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>12.348178137651832</v>
       </c>
       <c r="R111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>7.9185520361990891</v>
       </c>
       <c r="S111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>7.4340527577937854</v>
       </c>
       <c r="T111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>8.7947882736156391</v>
       </c>
       <c r="U111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>9.8198198198198305</v>
       </c>
       <c r="V111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>9.1544374563242492</v>
       </c>
       <c r="W111" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>10.342261904761907</v>
       </c>
     </row>
@@ -14512,83 +14512,83 @@
         <v>129</v>
       </c>
       <c r="J112" s="14">
-        <f t="shared" ref="J112:W112" si="13">J111</f>
+        <f t="shared" ref="J112:W112" si="14">J111</f>
         <v>18.609206660137122</v>
       </c>
       <c r="K112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>10.993249758919955</v>
       </c>
       <c r="L112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>13.54062186559679</v>
       </c>
       <c r="M112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>12.01814058956916</v>
       </c>
       <c r="N112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>9.4962840627580434</v>
       </c>
       <c r="O112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>8.6880973066898459</v>
       </c>
       <c r="P112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>8.4805653710247277</v>
       </c>
       <c r="Q112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>12.348178137651832</v>
       </c>
       <c r="R112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>7.9185520361990891</v>
       </c>
       <c r="S112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>7.4340527577937854</v>
       </c>
       <c r="T112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>8.7947882736156391</v>
       </c>
       <c r="U112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>9.8198198198198305</v>
       </c>
       <c r="V112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>9.1544374563242492</v>
       </c>
       <c r="W112" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>10.342261904761907</v>
       </c>
       <c r="X112" s="14">
-        <f t="shared" ref="X112:AC112" si="14">X83</f>
+        <f t="shared" ref="X112:AC112" si="15">X83</f>
         <v>9.1999999999999993</v>
       </c>
       <c r="Y112" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>7.2710000000000008</v>
       </c>
       <c r="Z112" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>7.82</v>
       </c>
       <c r="AA112" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>5.7200000000000006</v>
       </c>
       <c r="AB112" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>6.093</v>
       </c>
       <c r="AC112" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>5.9289999999999994</v>
       </c>
     </row>
@@ -14610,83 +14610,83 @@
         <v>131</v>
       </c>
       <c r="J114" s="14">
-        <f t="shared" ref="J114:W114" si="15">J24</f>
+        <f t="shared" ref="J114:W114" si="16">J24</f>
         <v>18.254834417332908</v>
       </c>
       <c r="K114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>12.735554542258573</v>
       </c>
       <c r="L114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>10.844222313156116</v>
       </c>
       <c r="M114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>11.902934481343165</v>
       </c>
       <c r="N114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>11.101183507729484</v>
       </c>
       <c r="O114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>8.9367511429333923</v>
       </c>
       <c r="P114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>8.8345878659570367</v>
       </c>
       <c r="Q114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>9.2584143379198842</v>
       </c>
       <c r="R114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>8.9185529153815679</v>
       </c>
       <c r="S114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>8.7399130223282189</v>
       </c>
       <c r="T114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>7.9366201773395595</v>
       </c>
       <c r="U114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>9.4827430112815936</v>
       </c>
       <c r="V114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>9.9559060617044448</v>
       </c>
       <c r="W114" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>8.7900177472390268</v>
       </c>
       <c r="X114" s="14">
-        <f t="shared" ref="X114:AC114" si="16">X85</f>
+        <f t="shared" ref="X114:AC114" si="17">X85</f>
         <v>8.9180921393257169</v>
       </c>
       <c r="Y114" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>7.2710000000000008</v>
       </c>
       <c r="Z114" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>7.82</v>
       </c>
       <c r="AA114" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>5.7200000000000006</v>
       </c>
       <c r="AB114" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>6.093</v>
       </c>
       <c r="AC114" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>5.9289999999999994</v>
       </c>
     </row>
@@ -18726,7 +18726,7 @@
         <v>219</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="K63" s="11">
         <v>0.46262529435054928</v>
@@ -19018,7 +19018,7 @@
         <v>226</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="K67" s="15">
         <f t="shared" ref="K67:X67" si="15">K66-K72</f>
@@ -19398,7 +19398,7 @@
         <v>235</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="K74" s="17">
         <f t="shared" ref="K74:X74" si="17">K60</f>
@@ -19880,7 +19880,7 @@
         <v>253</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="Y93" s="37">
         <f>Y174</f>
@@ -19976,7 +19976,7 @@
         <v>258</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="Y96" s="35">
         <v>0.99870147577222557</v>
@@ -20396,7 +20396,7 @@
     </row>
     <row r="112" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A112" s="40" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C112" s="35">
         <v>-0.40607077138265651</v>
@@ -20413,7 +20413,7 @@
     </row>
     <row r="113" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A113" s="40" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C113" s="35">
         <v>175.66233929374312</v>
@@ -20430,7 +20430,7 @@
     </row>
     <row r="114" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A114" s="40" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C114" s="35">
         <v>2.9586653733694201</v>
@@ -20466,7 +20466,7 @@
     </row>
     <row r="118" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A118" s="41" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
@@ -20503,24 +20503,24 @@
         <v>279</v>
       </c>
       <c r="B119" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="C119" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="C119" s="2" t="s">
+      <c r="F119" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="F119" s="2" t="s">
+      <c r="I119" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="I119" s="2" t="s">
+      <c r="L119" s="2" t="s">
         <v>283</v>
-      </c>
-      <c r="L119" s="2" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="120" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A120" s="40" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C120" s="35">
         <v>2.9586653733694201</v>
@@ -20529,7 +20529,8 @@
         <v>175.66233929374312</v>
       </c>
       <c r="E120" s="35">
-        <v>25.787231408321489</v>
+        <f>Income_Statement!$P$4*D120/1000</f>
+        <v>25.627589474371337</v>
       </c>
       <c r="F120" s="35">
         <v>2.4267920781857986</v>
@@ -20538,7 +20539,8 @@
         <v>170.95631606738016</v>
       </c>
       <c r="H120" s="35">
-        <v>22.532042457680703</v>
+        <f>Income_Statement!$Q$4*G120/1000</f>
+        <v>22.354820421673139</v>
       </c>
       <c r="I120" s="35">
         <v>0.95228762785498555</v>
@@ -20547,7 +20549,8 @@
         <v>187.90967275431009</v>
       </c>
       <c r="K120" s="35">
-        <v>31.760492888933499</v>
+        <f>Income_Statement!$R$4*J120/1000</f>
+        <v>31.646777471369493</v>
       </c>
       <c r="L120" s="35">
         <v>1.4419335507995614</v>
@@ -20556,12 +20559,13 @@
         <v>185.59485472528613</v>
       </c>
       <c r="N120" s="35">
-        <v>29.156951677342452</v>
+        <f>Income_Statement!$S$4*M120/1000</f>
+        <v>29.098073565629399</v>
       </c>
     </row>
     <row r="121" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A121" s="40" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C121" s="35">
         <v>2.9214530173966877</v>
@@ -20570,7 +20574,8 @@
         <v>175.59859824919744</v>
       </c>
       <c r="E121" s="35">
-        <v>25.777874222982188</v>
+        <f>Income_Statement!$P$4*D121/1000</f>
+        <v>25.618290216893314</v>
       </c>
       <c r="F121" s="35">
         <v>2.3799912087150075</v>
@@ -20579,7 +20584,8 @@
         <v>170.87791993092966</v>
       </c>
       <c r="H121" s="35">
-        <v>22.521709846896531</v>
+        <f>Income_Statement!$Q$4*G121/1000</f>
+        <v>22.344569080322213</v>
       </c>
       <c r="I121" s="35">
         <v>0.89734089758012525</v>
@@ -20588,7 +20594,8 @@
         <v>187.8070212728106</v>
       </c>
       <c r="K121" s="35">
-        <v>31.743142735530451</v>
+        <f>Income_Statement!$R$4*J121/1000</f>
+        <v>31.629489438536993</v>
       </c>
       <c r="L121" s="35">
         <v>1.3772666209542519</v>
@@ -20597,12 +20604,13 @@
         <v>185.47604217508132</v>
       </c>
       <c r="N121" s="35">
-        <v>29.138286225705279</v>
+        <f>Income_Statement!$S$4*M121/1000</f>
+        <v>29.079445806085651</v>
       </c>
     </row>
     <row r="122" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A122" s="40" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C122" s="35">
         <v>3.1846992445579829</v>
@@ -20611,7 +20619,8 @@
         <v>176.04951271170199</v>
       </c>
       <c r="E122" s="35">
-        <v>25.844068466077854</v>
+        <f>Income_Statement!$P$4*D122/1000</f>
+        <v>25.684074668925458</v>
       </c>
       <c r="F122" s="35">
         <v>2.6210779845884851</v>
@@ -20620,7 +20629,8 @@
         <v>171.2817643891953</v>
       </c>
       <c r="H122" s="35">
-        <v>22.574936546495945</v>
+        <f>Income_Statement!$Q$4*G122/1000</f>
+        <v>22.397377134160116</v>
       </c>
       <c r="I122" s="35">
         <v>1.1826561293439526</v>
@@ -20629,7 +20639,8 @@
         <v>188.3400471887918</v>
       </c>
       <c r="K122" s="35">
-        <v>31.833234775849597</v>
+        <f>Income_Statement!$R$4*J122/1000</f>
+        <v>31.719258912892819</v>
       </c>
       <c r="L122" s="35">
         <v>1.5629776027981197</v>
@@ -20638,12 +20649,13 @@
         <v>185.81724896202309</v>
       </c>
       <c r="N122" s="35">
-        <v>29.191889811933827</v>
+        <f>Income_Statement!$S$4*M122/1000</f>
+        <v>29.132941147873112</v>
       </c>
     </row>
     <row r="123" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A123" s="40" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C123" s="35">
         <v>2.5401382516811641</v>
@@ -20652,7 +20664,8 @@
         <v>174.94544418700329</v>
       </c>
       <c r="E123" s="35">
-        <v>25.681991206652089</v>
+        <f>Income_Statement!$P$4*D123/1000</f>
+        <v>25.523000786974936</v>
       </c>
       <c r="F123" s="35">
         <v>2.0157204261844122</v>
@@ -20661,7 +20674,8 @@
         <v>170.26772994311264</v>
       </c>
       <c r="H123" s="35">
-        <v>22.441286806502248</v>
+        <f>Income_Statement!$Q$4*G123/1000</f>
+        <v>22.264778593988989</v>
       </c>
       <c r="I123" s="35">
         <v>0.47744221353651828</v>
@@ -20670,7 +20684,8 @@
         <v>187.02256655128036</v>
       </c>
       <c r="K123" s="35">
-        <v>31.610554198497404</v>
+        <f>Income_Statement!$R$4*J123/1000</f>
+        <v>31.497375622123233</v>
       </c>
       <c r="L123" s="35">
         <v>1.0963357483499729</v>
@@ -20679,12 +20694,13 @@
         <v>184.95988788284552</v>
       </c>
       <c r="N123" s="35">
-        <v>29.057198386395029</v>
+        <f>Income_Statement!$S$4*M123/1000</f>
+        <v>28.998521711563075</v>
       </c>
     </row>
     <row r="124" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A124" s="40" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C124" s="35">
         <v>2.6034501079940413</v>
@@ -20693,7 +20709,8 @@
         <v>175.05389106568165</v>
       </c>
       <c r="E124" s="35">
-        <v>25.697911208442072</v>
+        <f>Income_Statement!$P$4*D124/1000</f>
+        <v>25.538822232241575</v>
       </c>
       <c r="F124" s="35">
         <v>1.6834657016993089</v>
@@ -20702,7 +20719,8 @@
         <v>169.71117005412765</v>
       </c>
       <c r="H124" s="35">
-        <v>22.367932213134026</v>
+        <f>Income_Statement!$Q$4*G124/1000</f>
+        <v>22.192000958986242</v>
       </c>
       <c r="I124" s="35">
         <v>0.86769862813263954</v>
@@ -20711,7 +20729,8 @@
         <v>187.75164358502883</v>
       </c>
       <c r="K124" s="35">
-        <v>31.733782798741569</v>
+        <f>Income_Statement!$R$4*J124/1000</f>
+        <v>31.620163014109657</v>
       </c>
       <c r="L124" s="35">
         <v>0.93734455107721582</v>
@@ -20720,12 +20739,13 @@
         <v>184.66777335609623</v>
       </c>
       <c r="N124" s="35">
-        <v>29.011307194242718</v>
+        <f>Income_Statement!$S$4*M124/1000</f>
+        <v>28.952723189823232</v>
       </c>
     </row>
     <row r="125" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A125" s="40" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C125" s="35">
         <v>3.4657406668111799</v>
@@ -20734,7 +20754,8 @@
         <v>176.53090856387951</v>
       </c>
       <c r="E125" s="35">
-        <v>25.914737377177516</v>
+        <f>Income_Statement!$P$4*D125/1000</f>
+        <v>25.75430608747466</v>
       </c>
       <c r="F125" s="35">
         <v>3.4657406668111799</v>
@@ -20743,7 +20764,8 @@
         <v>172.69665884818653</v>
       </c>
       <c r="H125" s="35">
-        <v>22.761419636190983</v>
+        <f>Income_Statement!$Q$4*G125/1000</f>
+        <v>22.582393472099351</v>
       </c>
       <c r="I125" s="35">
         <v>1.5267969042065266</v>
@@ -20752,7 +20774,8 @@
         <v>188.98297098438999</v>
       </c>
       <c r="K125" s="35">
-        <v>31.941901755781604</v>
+        <f>Income_Statement!$R$4*J125/1000</f>
+        <v>31.827536821060683</v>
       </c>
       <c r="L125" s="35">
         <v>1.4767969042065263</v>
@@ -20761,12 +20784,13 @@
         <v>185.65890916450081</v>
       </c>
       <c r="N125" s="35">
-        <v>29.167014629743068</v>
+        <f>Income_Statement!$S$4*M125/1000</f>
+        <v>29.108116197399731</v>
       </c>
     </row>
     <row r="126" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A126" s="40" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C126" s="35">
         <v>2.9586653733694201</v>
@@ -20775,7 +20799,8 @@
         <v>175.66233929374312</v>
       </c>
       <c r="E126" s="35">
-        <v>25.787231408321489</v>
+        <f>Income_Statement!$P$4*D126/1000</f>
+        <v>25.627589474371337</v>
       </c>
       <c r="F126" s="35">
         <v>2.4267920781857986</v>
@@ -20784,7 +20809,8 @@
         <v>170.95631606738016</v>
       </c>
       <c r="H126" s="35">
-        <v>22.532042457680703</v>
+        <f>Income_Statement!$Q$4*G126/1000</f>
+        <v>22.354820421673139</v>
       </c>
       <c r="I126" s="35">
         <v>1.5190733421406994</v>
@@ -20793,7 +20819,8 @@
         <v>188.96854182573867</v>
       </c>
       <c r="K126" s="35">
-        <v>31.939462939386349</v>
+        <f>Income_Statement!$R$4*J126/1000</f>
+        <v>31.825106736615087</v>
       </c>
       <c r="L126" s="35">
         <v>1.3187192650852757</v>
@@ -20802,12 +20829,13 @@
         <v>185.36847311814327</v>
       </c>
       <c r="N126" s="35">
-        <v>29.121387126860306</v>
+        <f>Income_Statement!$S$4*M126/1000</f>
+        <v>29.062580832448308</v>
       </c>
     </row>
     <row r="127" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A127" s="40" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C127" s="35">
         <v>1.4316998859615553</v>
@@ -20816,7 +20844,8 @@
         <v>173.0468001103622</v>
       </c>
       <c r="E127" s="35">
-        <v>25.403270256201171</v>
+        <f>Income_Statement!$P$4*D127/1000</f>
+        <v>25.246005324260874</v>
       </c>
       <c r="F127" s="35">
         <v>0.89982659077793359</v>
@@ -20825,7 +20854,8 @@
         <v>168.39849617942326</v>
       </c>
       <c r="H127" s="35">
-        <v>22.194921796447986</v>
+        <f>Income_Statement!$Q$4*G127/1000</f>
+        <v>22.020351326985093</v>
       </c>
       <c r="I127" s="35">
         <v>0.78553161653915915</v>
@@ -20834,7 +20864,8 @@
         <v>187.59813917396983</v>
       </c>
       <c r="K127" s="35">
-        <v>31.707837483184388</v>
+        <f>Income_Statement!$R$4*J127/1000</f>
+        <v>31.594310593281861</v>
       </c>
       <c r="L127" s="35">
         <v>1.275177539483735</v>
@@ -20843,12 +20874,13 @@
         <v>185.28847390569561</v>
       </c>
       <c r="N127" s="35">
-        <v>29.108819250584776</v>
+        <f>Income_Statement!$S$4*M127/1000</f>
+        <v>29.050038335122935</v>
       </c>
     </row>
     <row r="128" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A128" s="40" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C128" s="35">
         <v>2.2160130582524169</v>
@@ -20857,7 +20889,8 @@
         <v>174.39025014317923</v>
       </c>
       <c r="E128" s="35">
-        <v>25.60048872101871</v>
+        <f>Income_Statement!$P$4*D128/1000</f>
+        <v>25.442002861688589</v>
       </c>
       <c r="F128" s="35">
         <v>1.3388105403602899</v>
@@ -20866,7 +20899,8 @@
         <v>169.13383819336866</v>
       </c>
       <c r="H128" s="35">
-        <v>22.291839873885991</v>
+        <f>Income_Statement!$Q$4*G128/1000</f>
+        <v>22.116507111388998</v>
       </c>
       <c r="I128" s="35">
         <v>1.0639393858161017</v>
@@ -20875,7 +20909,8 @@
         <v>188.11826056853303</v>
       </c>
       <c r="K128" s="35">
-        <v>31.795748401293459</v>
+        <f>Income_Statement!$R$4*J128/1000</f>
+        <v>31.681906754727798</v>
       </c>
       <c r="L128" s="35">
         <v>1.4789182722462451</v>
@@ -20884,12 +20919,13 @@
         <v>185.66280675400009</v>
       </c>
       <c r="N128" s="35">
-        <v>29.16762694105342</v>
+        <f>Income_Statement!$S$4*M128/1000</f>
+        <v>29.108727272238774</v>
       </c>
     </row>
     <row r="129" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A129" s="40" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C129" s="35">
         <v>3.1301653733694201</v>
@@ -20898,7 +20934,8 @@
         <v>175.95610164374312</v>
       </c>
       <c r="E129" s="35">
-        <v>25.83035572130149</v>
+        <f>Income_Statement!$P$4*D129/1000</f>
+        <v>25.670446816127658</v>
       </c>
       <c r="F129" s="35">
         <v>2.8012920781857984</v>
@@ -20907,7 +20944,8 @@
         <v>171.58364101738019</v>
       </c>
       <c r="H129" s="35">
-        <v>22.614723886090708</v>
+        <f>Income_Statement!$Q$4*G129/1000</f>
+        <v>22.436851533046401</v>
       </c>
       <c r="I129" s="35">
         <v>1.2973876278549854</v>
@@ -20916,7 +20954,8 @@
         <v>188.55438857431008</v>
       </c>
       <c r="K129" s="35">
-        <v>31.869462756829893</v>
+        <f>Income_Statement!$R$4*J129/1000</f>
+        <v>31.75535718304026</v>
       </c>
       <c r="L129" s="35">
         <v>1.7527335507995614</v>
@@ -20925,12 +20964,13 @@
         <v>186.16588756528611</v>
       </c>
       <c r="N129" s="35">
-        <v>29.246660936506451</v>
+        <f>Income_Statement!$S$4*M129/1000</f>
+        <v>29.187601670335237</v>
       </c>
     </row>
     <row r="131" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A131" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B131" s="4"/>
       <c r="C131" s="4"/>
@@ -20964,34 +21004,34 @@
     </row>
     <row r="132" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A132" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="C132" s="3" t="s">
         <v>295</v>
-      </c>
-      <c r="C132" s="3" t="s">
-        <v>296</v>
       </c>
       <c r="D132" s="11">
         <v>-0.45338504985103428</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F132" s="11">
         <v>-0.151696241914275</v>
       </c>
       <c r="G132" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H132" s="11">
         <v>-0.1372192626177384</v>
       </c>
       <c r="I132" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J132" s="11">
         <v>-0.1468077761157966</v>
       </c>
       <c r="K132" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="L132" s="11">
         <v>-0.24</v>
@@ -20999,22 +21039,22 @@
     </row>
     <row r="133" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A133" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="C133" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="C133" s="3" t="s">
-        <v>302</v>
       </c>
       <c r="D133" s="11">
         <v>0.90892173109817698</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F133" s="11">
         <v>0.71904902180125252</v>
       </c>
       <c r="G133" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H133" s="11">
         <v>0.75</v>
@@ -21022,34 +21062,34 @@
     </row>
     <row r="134" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A134" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="C134" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="C134" s="3" t="s">
-        <v>306</v>
       </c>
       <c r="D134" s="11">
         <v>1.127000224086993</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F134" s="11">
         <v>4.2238488378822402E-2</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H134" s="11">
         <v>0.34856954589133587</v>
       </c>
       <c r="I134" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J134" s="11">
         <v>1.9054309022826501</v>
       </c>
       <c r="K134" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="L134" s="11">
         <v>23</v>
@@ -21057,28 +21097,28 @@
     </row>
     <row r="135" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A135" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="C135" s="3" t="s">
         <v>311</v>
-      </c>
-      <c r="C135" s="3" t="s">
-        <v>312</v>
       </c>
       <c r="D135" s="11">
         <v>-0.30222502486966091</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F135" s="11">
         <v>1.2350241649067231</v>
       </c>
       <c r="G135" s="3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H135" s="11">
         <v>1.127000224086993</v>
       </c>
       <c r="I135" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J135" s="11">
         <v>1.2472778236066191</v>
@@ -21086,16 +21126,16 @@
     </row>
     <row r="136" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A136" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="C136" s="3" t="s">
         <v>316</v>
-      </c>
-      <c r="C136" s="3" t="s">
-        <v>317</v>
       </c>
       <c r="D136" s="11">
         <v>1.0851967961560449</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F136" s="11">
         <v>-0.3813639149721989</v>
@@ -21103,28 +21143,28 @@
     </row>
     <row r="137" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A137" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="C137" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="C137" s="3" t="s">
-        <v>320</v>
       </c>
       <c r="D137" s="11">
         <v>2.9526845695360309</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F137" s="11">
         <v>2.7541152323978588</v>
       </c>
       <c r="G137" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H137" s="11">
         <v>2.9342351202074228</v>
       </c>
       <c r="I137" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J137" s="11">
         <v>0.73948141424267821</v>
@@ -21132,28 +21172,28 @@
     </row>
     <row r="138" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A138" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D138" s="11">
         <v>3.2582814816847372</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F138" s="11">
         <v>2.6850302492115929</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H138" s="11">
         <v>2.6789213514875398</v>
       </c>
       <c r="I138" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J138" s="11">
         <v>0.73948141424267821</v>
@@ -21161,28 +21201,28 @@
     </row>
     <row r="139" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A139" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D139" s="11">
         <v>3.3394495262007751</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F139" s="11">
         <v>3.1536917790815262</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H139" s="11">
         <v>3.9250552425077929</v>
       </c>
       <c r="I139" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J139" s="11">
         <v>-0.25133870805769121</v>
@@ -21190,16 +21230,16 @@
     </row>
     <row r="140" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A140" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="C140" s="3" t="s">
         <v>326</v>
-      </c>
-      <c r="C140" s="3" t="s">
-        <v>327</v>
       </c>
       <c r="D140" s="11">
         <v>0.42</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F140" s="11">
         <v>1.29</v>
@@ -21207,40 +21247,40 @@
     </row>
     <row r="141" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A141" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="C141" s="3" t="s">
         <v>329</v>
-      </c>
-      <c r="C141" s="3" t="s">
-        <v>330</v>
       </c>
       <c r="D141" s="11">
         <v>8.2894006196326794E-2</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F141" s="11">
         <v>0.7940309342115639</v>
       </c>
       <c r="G141" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H141" s="11">
         <v>-0.53940323286848835</v>
       </c>
       <c r="I141" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J141" s="11">
         <v>0.70519124526114219</v>
       </c>
       <c r="K141" s="3" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="L141" s="11">
         <v>94</v>
       </c>
       <c r="M141" s="3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="N141" s="11">
         <v>4.1103455300918003E-2</v>
@@ -21248,40 +21288,40 @@
     </row>
     <row r="142" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A142" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="C142" s="3" t="s">
         <v>336</v>
-      </c>
-      <c r="C142" s="3" t="s">
-        <v>337</v>
       </c>
       <c r="D142" s="11">
         <v>81.044074742800262</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F142" s="11">
         <v>39.955891630212349</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H142" s="11">
         <v>62.94056049407353</v>
       </c>
       <c r="I142" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J142" s="11">
         <v>56.764629864682753</v>
       </c>
       <c r="K142" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="L142" s="11">
         <v>0.86565006300823488</v>
       </c>
       <c r="M142" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="N142" s="11">
         <v>-0.34492205676658533</v>
@@ -21289,7 +21329,7 @@
     </row>
     <row r="145" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A145" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="O145" s="19">
         <f t="shared" ref="O145:AD145" si="28">O6</f>
@@ -21358,7 +21398,7 @@
     </row>
     <row r="146" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A146" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="Y146" s="19">
         <f>Y99</f>
@@ -21371,7 +21411,7 @@
     </row>
     <row r="147" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A147" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="O147" s="19">
         <f t="shared" ref="O147:AD147" si="29">O50</f>
@@ -21440,7 +21480,7 @@
     </row>
     <row r="148" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A148" s="7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="O148" s="19">
         <f t="shared" ref="O148:X148" si="30">O9</f>
@@ -21485,7 +21525,7 @@
     </row>
     <row r="168" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A168" s="41" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B168" s="43"/>
       <c r="C168" s="43"/>
@@ -21519,10 +21559,10 @@
     </row>
     <row r="169" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A169" s="44" t="s">
+        <v>395</v>
+      </c>
+      <c r="B169" s="45" t="s">
         <v>396</v>
-      </c>
-      <c r="B169" s="45" t="s">
-        <v>397</v>
       </c>
       <c r="Y169" s="11">
         <v>-0.2981160231923986</v>
@@ -21545,10 +21585,10 @@
     </row>
     <row r="170" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A170" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="B170" s="45" t="s">
         <v>398</v>
-      </c>
-      <c r="B170" s="45" t="s">
-        <v>399</v>
       </c>
       <c r="X170" s="11">
         <v>-0.05</v>
@@ -21556,10 +21596,10 @@
     </row>
     <row r="171" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A171" s="44" t="s">
+        <v>399</v>
+      </c>
+      <c r="B171" s="45" t="s">
         <v>400</v>
-      </c>
-      <c r="B171" s="45" t="s">
-        <v>401</v>
       </c>
       <c r="Y171" s="11">
         <v>0</v>
@@ -21582,10 +21622,10 @@
     </row>
     <row r="172" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A172" s="44" t="s">
+        <v>401</v>
+      </c>
+      <c r="B172" s="45" t="s">
         <v>402</v>
-      </c>
-      <c r="B172" s="45" t="s">
-        <v>403</v>
       </c>
       <c r="X172" s="15">
         <f>(SUM(K67:X67)+X170)/COUNT(K67:X67)</f>
@@ -21594,10 +21634,10 @@
     </row>
     <row r="173" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A173" s="44" t="s">
+        <v>403</v>
+      </c>
+      <c r="B173" s="45" t="s">
         <v>404</v>
-      </c>
-      <c r="B173" s="45" t="s">
-        <v>405</v>
       </c>
       <c r="Y173" s="11">
         <v>-1.2274229593900643</v>
@@ -21608,10 +21648,10 @@
     </row>
     <row r="174" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A174" s="44" t="s">
+        <v>405</v>
+      </c>
+      <c r="B174" s="45" t="s">
         <v>406</v>
-      </c>
-      <c r="B174" s="45" t="s">
-        <v>407</v>
       </c>
       <c r="Y174" s="15">
         <f>(Y50+Y173)/2</f>
@@ -21624,10 +21664,10 @@
     </row>
     <row r="175" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A175" s="44" t="s">
+        <v>407</v>
+      </c>
+      <c r="B175" s="45" t="s">
         <v>408</v>
-      </c>
-      <c r="B175" s="45" t="s">
-        <v>409</v>
       </c>
       <c r="Y175" s="11">
         <v>2.9567729500361201E-2</v>
@@ -21650,10 +21690,10 @@
     </row>
     <row r="176" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A176" s="44" t="s">
+        <v>409</v>
+      </c>
+      <c r="B176" s="45" t="s">
         <v>410</v>
-      </c>
-      <c r="B176" s="45" t="s">
-        <v>411</v>
       </c>
       <c r="Y176" s="14">
         <f t="shared" ref="Y176:AD176" si="31">U6*(1+(Y74+Y175)/100)</f>
@@ -21682,10 +21722,10 @@
     </row>
     <row r="177" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A177" s="44" t="s">
+        <v>411</v>
+      </c>
+      <c r="B177" s="45" t="s">
         <v>412</v>
-      </c>
-      <c r="B177" s="45" t="s">
-        <v>413</v>
       </c>
       <c r="Y177" s="14">
         <f t="shared" ref="Y177:AD177" si="32">U6*(1+(Y74+Y50)/100)</f>
@@ -21714,10 +21754,10 @@
     </row>
     <row r="178" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A178" s="44" t="s">
+        <v>413</v>
+      </c>
+      <c r="B178" s="45" t="s">
         <v>414</v>
-      </c>
-      <c r="B178" s="45" t="s">
-        <v>415</v>
       </c>
       <c r="Y178" s="10">
         <v>175.66233929374312</v>
@@ -21740,10 +21780,10 @@
     </row>
     <row r="179" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A179" s="44" t="s">
+        <v>415</v>
+      </c>
+      <c r="B179" s="45" t="s">
         <v>416</v>
-      </c>
-      <c r="B179" s="45" t="s">
-        <v>417</v>
       </c>
       <c r="Y179" s="14">
         <f t="shared" ref="Y179:AD179" si="33">Y95-Y178</f>

</xml_diff>